<commit_message>
data: fechamento completo da semana 21 a 27/09 e recuperacao de 100 lojas pendentes via varredura pwr
</commit_message>
<xml_diff>
--- a/dados_all_stores/KEYS Service Exceptions - All Stores (Stores) (2026-08-30).xlsx
+++ b/dados_all_stores/KEYS Service Exceptions - All Stores (Stores) (2026-08-30).xlsx
@@ -935,19 +935,19 @@
     <t>214</t>
   </si>
   <si>
-    <t>21</t>
+    <t>20</t>
   </si>
   <si>
-    <t>R$ 8.920,77</t>
+    <t>R$ 8.934,66</t>
   </si>
   <si>
-    <t>97.5</t>
+    <t>97.7</t>
   </si>
   <si>
     <t>64.3</t>
   </si>
   <si>
-    <t>6.70</t>
+    <t>6.69</t>
   </si>
   <si>
     <t>21.5</t>
@@ -959,7 +959,7 @@
     <t>6.4</t>
   </si>
   <si>
-    <t>32.4%</t>
+    <t>32.7%</t>
   </si>
   <si>
     <t>16.1%</t>
@@ -10127,7 +10127,7 @@
         <v>19618</v>
       </c>
       <c r="B58" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C58" s="4">
         <v>51</v>
@@ -10157,18 +10157,30 @@
         <v>58</v>
       </c>
       <c r="L58" s="4"/>
-      <c r="M58" s="5"/>
-      <c r="N58" s="6"/>
+      <c r="M58" s="5">
+        <v>11573.209999999999</v>
+      </c>
+      <c r="N58" s="6">
+        <v>132</v>
+      </c>
       <c r="O58" s="6">
         <v>102</v>
       </c>
-      <c r="P58" s="7"/>
-      <c r="Q58" s="8"/>
-      <c r="R58" s="8"/>
+      <c r="P58" s="7">
+        <v>4.4328162790697672</v>
+      </c>
+      <c r="Q58" s="8">
+        <v>17.740196078431371</v>
+      </c>
+      <c r="R58" s="8">
+        <v>6.2412544554455449</v>
+      </c>
       <c r="S58" s="8">
         <v>7</v>
       </c>
-      <c r="T58" s="9"/>
+      <c r="T58" s="9">
+        <v>0.37254901960784315</v>
+      </c>
       <c r="U58" s="9">
         <v>0.11764705882352941</v>
       </c>

</xml_diff>